<commit_message>
Reclassify nuts to 7318 16 99; remove antidumping flag
Per previous Sonavox declaration, the nuts go to 7318 16 99 (matice),
not 7318 15 95 19. Nuts are outside the scope of Reg. (EU) 2022/191
(scope covers wood screws, self-tapping screws, other screws and bolts
with heads, and washers) and no line of the 7318 16 tree carries a
KDUMP/CDUMP marker in the Czech ECIT chapter 73 tariff. Sonavox's own
HS list corroborates: 3,70 % on Insert (nut) vs 3,7 + 86,5 % on SCREW.

Row keeps its CBAM flag (heading 7318 is in CBAM Annex I, receiver
Y137). Open points recorded: internal diameter (7318 16 91 vs 99),
the "AL" in part 029-2513-AL-CZ, and the spring nut.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016aE9TNqsBNtBLAxXd4cMbQ
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonavox_TECGO26080180.xlsx
+++ b/output/HS_Code_Summary_Sonavox_TECGO26080180.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dokumenty a poznámky" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dokumenty a poznámky" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,7 +55,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
+        <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -754,12 +754,12 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>7318159519</t>
+          <t>73181699</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Matice a pružná matice (nut, spring nut) – spojovací materiál ze železa nebo oceli</t>
+          <t>Matice a pružná matice (nut, spring nut) – matice ze železa nebo oceli, vnitřní průměr převyšující 12 mm</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -786,12 +786,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>CBAM + ANTIDUMPING</t>
+          <t>CBAM</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>CBAM zboží (železo/ocel), 961,14 kg NW – příjemce Sonavox Technology CZ s.r.o. má v registru kód Y137 (de minimis, do 50 t/rok). ANTIDUMPING: spojovací materiál ze železa/oceli z ČLR – nař. (EU) 2022/191, zbytková sazba 86,5 % + clo 3,7 %. POZOR: díl 029-2513-AL-CZ má v označení 'AL' (hliník) – pokud jde o hliník, zařazení 7318 (ocel) neplatí. Ověřit materiál u odesílatele.</t>
+          <t>Kód dle předchozí deklarace Sonavox. TARIC 10 míst: 7318169999 (Ostatní), clo 3,7 %. BEZ ANTIDUMPINGU – matice (7318 16) nejsou v rozsahu nař. (EU) 2022/191; v ECIT kap. 73 nemá žádný řádek 7318 16 značku KDUMP/CDUMP. Sazebník SONAVOX to potvrzuje: u Insert (nut) uvádí jen 3,70 %, u SCREW 3,7 + 86,5 %. CBAM zboží (železo/ocel, hlava 7318 je v příloze I CBAM), 961,14 kg NW – příjemce má kód Y137 (de minimis, do 50 t/rok). K OVĚŘENÍ: (1) vnitřní průměr – při ≤ 12 mm patří do 7318 16 91 (7318169199), ne ...99; hmotnost 1,665 g/ks nasvědčuje malé matici. (2) díl 029-2513-AL-CZ má v označení 'AL' (hliník) – hliníková matice nepatří do 7318, ale do 7616 10 00 (CBAM zůstává). (3) pružná matice 029A-000004-CZ (0,42 g/ks) – ověřit, zda jde rovněž o matici 7318 16.</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>Antidumpingové clo – nutno zkontrolovat a uvést v JSD (zde současně i CBAM).</t>
+          <t>Antidumpingové clo – v této zásilce se neuplatňuje žádná položka (viz list Dokumenty a poznámky).</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1078,14 +1078,14 @@
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>→ Do JSD uvést kód Y137 (výjimka de minimis, dovoz do 50 t/rok) u položky 7318 1595 19.</t>
+          <t>→ Do JSD uvést kód Y137 (výjimka de minimis, dovoz do 50 t/rok) u položky 7318 16 99.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Dotčené CBAM zboží v zásilce: 7318 1595 19 (matice, železo/ocel) – 961,14 kg NW. Ostatní položky (8518, 8504, 3926, 7409) pod CBAM nespadají.</t>
+          <t>Dotčené CBAM zboží v zásilce: 7318 16 99 (matice, železo/ocel) – 961,14 kg NW. Ostatní položky (8518, 8504, 3926, 7409) pod CBAM nespadají.</t>
         </is>
       </c>
     </row>
@@ -1108,162 +1108,211 @@
     </row>
     <row r="22">
       <c r="A22" s="18">
-        <f>== ANTIDUMPING – 7318 1595 19 (matice, ČLR) ===</f>
+        <f>== ANTIDUMPING – NEUPLATŇUJE SE ===</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Spojovací materiál ze železa nebo oceli původem z ČLR podléhá antidumpingovému clu – prováděcí nařízení (EU) 2022/191.</t>
+          <t>Matice zařazeny do 7318 16 99 (kód dle předchozí deklarace Sonavox). Matice NEJSOU v rozsahu prováděcího nařízení (EU) 2022/191.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Zbytková sazba 86,5 % (sazebník SONAVOX u položky SCREW výslovně uvádí '3,7 + 86,5 %'), vedle smluvního cla 3,7 %.</t>
+          <t>Rozsah 2022/191: vruty do dřeva (mimo vrtule), samovrtné šrouby, ostatní šrouby a svorníky s hlavou a podložky.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Hodnota dotčeného zboží: 40 410,00 EUR (029-2513-AL-CZ 40 320,00 EUR + 029A-000004-CZ 90,00 EUR) → dopad je významný, ověřit sazbu a případný individuální kód doplňkového cla (TARIC) u výrobce před podáním JSD.</t>
+          <t>Pokryté kódy: 7318 12 90, 7318 14 91, 7318 14 99, 7318 15 58, 7318 15 68, 7318 15 82, 7318 15 88, ex 7318 15 95 (TARIC 7318159519 a 7318159589), ex 7318 21 00, ex 7318 22 00. Podpoložka 7318 16 (matice) v seznamu NENÍ.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>UPOZORNĚNÍ NA MATERIÁL: číslo dílu 029-2513-AL-CZ obsahuje 'AL'. Je-li matice hliníková, nepatří do 7318 (ocel) – pak neplatí antidumping, ale zboží zůstává CBAM (hliník je rovněž v příloze I CBAM). Nutné potvrzení materiálu od odesílatele.</t>
+          <t>Ověřeno v ECIT, kapitola 73 (celnisprava.gov.cz): žádný řádek stromu 7318 16 nenese značku KDUMP ani CDUMP; celní sazba 3,7 % pro třetí země.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr"/>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Naproti tomu řádky 7318 15 xx značku KDUMP nesou (a CDUMP u obcházení přes Malajsii / Filipíny).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="18">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Sazebník SONAVOX to potvrzuje: u položky 'Insert (nut)' uvádí pouze 3,70 %, kdežto u 'SCREW: šroub' uvádí '3,7 + 86,5 %'. Kód 7318159519 uvedený v sazebníku u matice je tedy kód pro šrouby/svorníky – nesprávně spárovaný se správnou sazbou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Pozn.: kdyby zařazení 7318 15 95 19 platilo, uplatnil by se přídavný kód C999 (všechny ostatní společnosti) se sazbou 86,5 %. Suzhou Sonavox International Trading Co., Ltd. není v příloze nař. 2022/191 (ta uvádí vyvážející výrobce spojovacího materiálu) a jde navíc o obchodní, nikoli výrobní společnost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>K OVĚŘENÍ – VNITŘNÍ PRŮMĚR: 7318 16 99 = vnitřní průměr převyšující 12 mm; 7318 16 91 = nepřesahující 12 mm. Hmotnost 029-2513-AL-CZ je 1,665 g/ks (576 000 ks / 959,04 kg), což nasvědčuje malé matici → prověřit, zda nepatří do 7318 16 91 (7318169199). Clo 3,7 % je v obou případech stejné, antidumping se neuplatní ani v jednom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>K OVĚŘENÍ – MATERIÁL: číslo dílu 029-2513-AL-CZ obsahuje 'AL'. Je-li matice hliníková, nepatří do 7318 (železo/ocel), ale do 7616 10 00 (sazebník SONAVOX používá tento kód pro Aluminium ring). CBAM platí i tak (hliník je rovněž v příloze I CBAM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>K OVĚŘENÍ – PRUŽNÁ MATICE: 029A-000004-CZ, 0,42 g/ks – ověřit, zda jde rovněž o matici 7318 16, nebo o výlisek z plechu (7326).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="18">
         <f>== COO / PREFERENČNÍ VĚTA – NENALEZENA ===</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>V žádném z dokladů (faktury CZ20260814 a CZ20260814-1, packing listy, FCR TECGO26080180) NENÍ uvedena preferenční věta o původu.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Uvedený původ zboží: Čína (Origin of Goods: China; u faktury CZ20260814-1 navíc 'Origin of Goods: Suzhou (35029)').</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Jediné prohlášení na fakturách je vývozní doložka ('THESE COMMODITIES ... EXPORTED FROM CHINA ...') – to není preferenční věta.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>→ ČLR nemá s EU preferenční dohodu, uplatní se plné smluvní clo třetí země. Preferenční sazbu nelze nárokovat.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="18">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="18">
         <f>== ZAŘAZENÍ – ZDROJ A ODVOZENÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>HS kódy vycházejí ze sazebníku komponent SONAVOX (e-mail 'Re: SONAVOX HS KODY', Ing. Michaela Ryan).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Matice: 7318 16 99 podle předchozí deklarace Sonavox (sazebník uvádí u Insert (nut) kód 7318159519 – pro matice nesprávný, viz sekce ANTIDUMPING).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>Přímo ze sazebníku: Voice coil → 8504 5000 00; Spider / Cone / T-yoke / Ceramics circle → 8518 9000 00; Gasket (plastové těsnění) → 3926 9097.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Odvozeno (v sazebníku není doslovně): Terminal → 7409 3900 ('Pin, lug / kontakt'); Nut a Spring nut → 7318 1595 19 ('Insert (nut)'). Obojí potvrdit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>Odvozeno: Terminal → 7409 3900 ('Pin, lug / kontakt'; v sazebníku není položka Terminal uvedena – zvážit i 8518 9000 00, viz níže). Potvrdit s odesílatelem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>U kódů 3926 9097 a 7409 3900 sazebník uvádí jen 8místný kód CN – doplnit TARIC (10 míst) při podání.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="18">
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="18">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>FOB Zhengzhou (Henan), CN.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>Termín FOB je převzat z obou faktur (Terms of Payment: FOB); místo doplněno z FCR (place of receipt / port of loading: ZHENGZHOU, HENAN). Přeprava je železniční (freight collect), FOB je původem námořní doložka – doporučuji potvrdit znění s odesílatelem.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="18">
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="18">
         <f>== SLEVA ===</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>Na fakturách není uvedena žádná obchodní sleva (Sub Total = Total Amount), proporcionální rozpočet slevy se neuplatňuje.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="18">
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="18">
         <f>== PODKLADY ===</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>HBL_TECGO26080180.pdf (FCR) · TRCZ20260814.xlsx (INV + PL, odesílatel A) · CIC001E260814002___GCS.xlsx (INV, odesílatel B) · PLC001E260814002___GCS.xlsx (PL, odesílatel B) · Re_SONAVOX_HS_KODY.eml (sazebník HS kódů)</t>
         </is>

</xml_diff>